<commit_message>
add groups and channel ids to biotek data
for fluorescence tests
</commit_message>
<xml_diff>
--- a/test/inputs/biotek.xlsx
+++ b/test/inputs/biotek.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4042B1F-748B-B646-9293-122223345008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBCEE06-64BB-F248-8523-377BEEB48EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19420" yWindow="7480" windowWidth="18980" windowHeight="9440" activeTab="4" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="19420" yWindow="7480" windowWidth="18980" windowHeight="9440" activeTab="2" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>Plate</t>
   </si>
@@ -100,6 +100,24 @@
   </si>
   <si>
     <t>View</t>
+  </si>
+  <si>
+    <t>flu1</t>
+  </si>
+  <si>
+    <t>485,530[2]</t>
+  </si>
+  <si>
+    <t>flu2</t>
+  </si>
+  <si>
+    <t>485,530</t>
+  </si>
+  <si>
+    <t>plate1</t>
+  </si>
+  <si>
+    <t>plate_01_[a:h][1:12]</t>
   </si>
 </sst>
 </file>
@@ -535,7 +553,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA707B9-0BE9-45E5-A5EE-A3873F0594F1}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -566,7 +584,20 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -575,7 +606,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D9B2676-373C-45A2-B753-09761E8A63AC}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -587,6 +618,14 @@
       </c>
       <c r="B1" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>